<commit_message>
Fix slot-aware transfers: slots are locked to players
Slots (D1/D2, I1/I2, C1/C2, S1/S2, W1-W3) are now fixed per player.
Transfers must respect slot role requirements — replacing a D slot
requires a duelist, wildcard slots accept any role. No more silently
moving players between slots without a transfer.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/VFL_2026_Stage1_Pricing.xlsx
+++ b/VFL_2026_Stage1_Pricing.xlsx
@@ -716,16 +716,16 @@
       </c>
       <c r="I6" s="7" t="inlineStr">
         <is>
-          <t>Lar0k</t>
+          <t>Derke</t>
         </is>
       </c>
       <c r="J6" s="7" t="inlineStr">
         <is>
-          <t>BBL Esports</t>
+          <t>Team Vitality</t>
         </is>
       </c>
       <c r="K6" s="7" t="n">
-        <v>9.5</v>
+        <v>12</v>
       </c>
       <c r="L6" s="7" t="n">
         <v>0</v>
@@ -762,12 +762,12 @@
       </c>
       <c r="I7" s="7" t="inlineStr">
         <is>
-          <t>Kushy</t>
+          <t>Sayonara</t>
         </is>
       </c>
       <c r="J7" s="7" t="inlineStr">
         <is>
-          <t>Rex Regum Qeon</t>
+          <t>Team Vitality</t>
         </is>
       </c>
       <c r="K7" s="7" t="n">
@@ -808,16 +808,16 @@
       </c>
       <c r="I8" s="7" t="inlineStr">
         <is>
-          <t>cloud</t>
+          <t>BeYN</t>
         </is>
       </c>
       <c r="J8" s="7" t="inlineStr">
         <is>
-          <t>GIANTX</t>
+          <t>DRX</t>
         </is>
       </c>
       <c r="K8" s="7" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="L8" s="7" t="n">
         <v>0</v>
@@ -900,16 +900,16 @@
       </c>
       <c r="I10" s="7" t="inlineStr">
         <is>
-          <t>xavi8k</t>
+          <t>crazyguy</t>
         </is>
       </c>
       <c r="J10" s="7" t="inlineStr">
         <is>
-          <t>Global Esports</t>
+          <t>Rex Regum Qeon</t>
         </is>
       </c>
       <c r="K10" s="7" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="L10" s="7" t="n">
         <v>0</v>
@@ -946,16 +946,16 @@
       </c>
       <c r="I11" s="7" t="inlineStr">
         <is>
-          <t>Meteor</t>
+          <t>caedye</t>
         </is>
       </c>
       <c r="J11" s="7" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>Detonation FocusMe</t>
         </is>
       </c>
       <c r="K11" s="7" t="n">
-        <v>12</v>
+        <v>8.5</v>
       </c>
       <c r="L11" s="7" t="n">
         <v>0</v>
@@ -992,16 +992,16 @@
       </c>
       <c r="I12" s="7" t="inlineStr">
         <is>
-          <t>echo</t>
+          <t>Westside</t>
         </is>
       </c>
       <c r="J12" s="7" t="inlineStr">
         <is>
-          <t>Eternal Fire</t>
+          <t>GIANTX</t>
         </is>
       </c>
       <c r="K12" s="7" t="n">
-        <v>5</v>
+        <v>7.5</v>
       </c>
       <c r="L12" s="7" t="n">
         <v>0</v>
@@ -1038,7 +1038,7 @@
       </c>
       <c r="I13" s="7" t="inlineStr">
         <is>
-          <t>Lovers rock</t>
+          <t>Lar0k</t>
         </is>
       </c>
       <c r="J13" s="7" t="inlineStr">
@@ -1047,7 +1047,7 @@
         </is>
       </c>
       <c r="K13" s="7" t="n">
-        <v>9</v>
+        <v>9.5</v>
       </c>
       <c r="L13" s="7" t="n">
         <v>0</v>
@@ -1084,16 +1084,16 @@
       </c>
       <c r="I14" s="7" t="inlineStr">
         <is>
-          <t>Jemkin</t>
+          <t>Lovers rock</t>
         </is>
       </c>
       <c r="J14" s="7" t="inlineStr">
         <is>
-          <t>Rex Regum Qeon</t>
+          <t>BBL Esports</t>
         </is>
       </c>
       <c r="K14" s="7" t="n">
-        <v>11.5</v>
+        <v>9</v>
       </c>
       <c r="L14" s="7" t="n">
         <v>0</v>
@@ -1130,16 +1130,16 @@
       </c>
       <c r="I15" s="7" t="inlineStr">
         <is>
-          <t>MrFalin</t>
+          <t>BuZz</t>
         </is>
       </c>
       <c r="J15" s="7" t="inlineStr">
         <is>
-          <t>FUT Esports</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="K15" s="7" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="L15" s="7" t="n">
         <v>0</v>
@@ -1169,14 +1169,14 @@
         </is>
       </c>
       <c r="J16" s="9" t="n">
-        <v>98.5</v>
+        <v>100</v>
       </c>
       <c r="L16" s="9" t="n">
-        <v>97.7</v>
+        <v>98</v>
       </c>
       <c r="M16" s="5" t="inlineStr">
         <is>
-          <t>IGL: 109.0</t>
+          <t>IGL: 109.3</t>
         </is>
       </c>
     </row>
@@ -1195,12 +1195,12 @@
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>Transfers: OUT PROFEK, Veqaj, BeYN -&gt; IN Dos9, LewN, xavi8k</t>
+          <t>Transfers: [W3] BeYN -&gt; xavi8k | [C2] PROFEK -&gt; Dos9 | [D1] xeus -&gt; LewN</t>
         </is>
       </c>
       <c r="H19" s="5" t="inlineStr">
         <is>
-          <t>Transfers: OUT MrFalin, Jemkin, Meteor -&gt; IN Autumn, LewN, skuba</t>
+          <t>Transfers: [D2] Derke -&gt; LewN | [I2] BeYN -&gt; N4RRATE | [I1] Sayonara -&gt; Kushy</t>
         </is>
       </c>
     </row>
@@ -1238,25 +1238,21 @@
       </c>
       <c r="I20" s="7" t="inlineStr">
         <is>
-          <t>LewN</t>
+          <t>xeus</t>
         </is>
       </c>
       <c r="J20" s="7" t="inlineStr">
         <is>
-          <t>Karmine Corp</t>
+          <t>FUT Esports</t>
         </is>
       </c>
       <c r="K20" s="7" t="n">
-        <v>11.5</v>
+        <v>9.5</v>
       </c>
       <c r="L20" s="7" t="n">
-        <v>12</v>
-      </c>
-      <c r="M20" s="8" t="inlineStr">
-        <is>
-          <t>IGL</t>
-        </is>
-      </c>
+        <v>9.800000000000001</v>
+      </c>
+      <c r="M20" s="7" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
@@ -1288,21 +1284,25 @@
       </c>
       <c r="I21" s="7" t="inlineStr">
         <is>
-          <t>Autumn</t>
+          <t>LewN</t>
         </is>
       </c>
       <c r="J21" s="7" t="inlineStr">
         <is>
-          <t>Global Esports</t>
+          <t>Karmine Corp</t>
         </is>
       </c>
       <c r="K21" s="7" t="n">
-        <v>8.5</v>
+        <v>11.5</v>
       </c>
       <c r="L21" s="7" t="n">
-        <v>11.1</v>
-      </c>
-      <c r="M21" s="7" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="M21" s="8" t="inlineStr">
+        <is>
+          <t>IGL</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
@@ -1380,19 +1380,19 @@
       </c>
       <c r="I23" s="7" t="inlineStr">
         <is>
-          <t>cloud</t>
+          <t>N4RRATE</t>
         </is>
       </c>
       <c r="J23" s="7" t="inlineStr">
         <is>
-          <t>GIANTX</t>
+          <t>Karmine Corp</t>
         </is>
       </c>
       <c r="K23" s="7" t="n">
-        <v>7</v>
+        <v>9.5</v>
       </c>
       <c r="L23" s="7" t="n">
-        <v>7.5</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="M23" s="7" t="inlineStr"/>
     </row>
@@ -1404,19 +1404,19 @@
       </c>
       <c r="B24" s="7" t="inlineStr">
         <is>
-          <t>xavi8k</t>
+          <t>Veqaj</t>
         </is>
       </c>
       <c r="C24" s="7" t="inlineStr">
         <is>
-          <t>Global Esports</t>
+          <t>FNATIC</t>
         </is>
       </c>
       <c r="D24" s="7" t="n">
-        <v>7.5</v>
+        <v>10.5</v>
       </c>
       <c r="E24" s="7" t="n">
-        <v>10.3</v>
+        <v>8.6</v>
       </c>
       <c r="F24" s="7" t="inlineStr"/>
       <c r="H24" s="6" t="inlineStr">
@@ -1426,19 +1426,19 @@
       </c>
       <c r="I24" s="7" t="inlineStr">
         <is>
-          <t>xavi8k</t>
+          <t>Veqaj</t>
         </is>
       </c>
       <c r="J24" s="7" t="inlineStr">
         <is>
-          <t>Global Esports</t>
+          <t>FNATIC</t>
         </is>
       </c>
       <c r="K24" s="7" t="n">
-        <v>9</v>
+        <v>9.5</v>
       </c>
       <c r="L24" s="7" t="n">
-        <v>10.3</v>
+        <v>8.6</v>
       </c>
       <c r="M24" s="7" t="inlineStr"/>
     </row>
@@ -1472,19 +1472,19 @@
       </c>
       <c r="I25" s="7" t="inlineStr">
         <is>
-          <t>Veqaj</t>
+          <t>crazyguy</t>
         </is>
       </c>
       <c r="J25" s="7" t="inlineStr">
         <is>
-          <t>FNATIC</t>
+          <t>Rex Regum Qeon</t>
         </is>
       </c>
       <c r="K25" s="7" t="n">
-        <v>9.5</v>
+        <v>5</v>
       </c>
       <c r="L25" s="7" t="n">
-        <v>8.6</v>
+        <v>5.7</v>
       </c>
       <c r="M25" s="7" t="inlineStr"/>
     </row>
@@ -1496,19 +1496,19 @@
       </c>
       <c r="B26" s="7" t="inlineStr">
         <is>
-          <t>Yetujey</t>
+          <t>Free1ng</t>
         </is>
       </c>
       <c r="C26" s="7" t="inlineStr">
         <is>
-          <t>FUT Esports</t>
+          <t>DRX</t>
         </is>
       </c>
       <c r="D26" s="7" t="n">
         <v>7.5</v>
       </c>
       <c r="E26" s="7" t="n">
-        <v>7.3</v>
+        <v>6.3</v>
       </c>
       <c r="F26" s="7" t="inlineStr"/>
       <c r="H26" s="6" t="inlineStr">
@@ -1518,19 +1518,19 @@
       </c>
       <c r="I26" s="7" t="inlineStr">
         <is>
-          <t>skuba</t>
+          <t>caedye</t>
         </is>
       </c>
       <c r="J26" s="7" t="inlineStr">
         <is>
-          <t>NRG Esports</t>
+          <t>Detonation FocusMe</t>
         </is>
       </c>
       <c r="K26" s="7" t="n">
-        <v>13</v>
+        <v>8.5</v>
       </c>
       <c r="L26" s="7" t="n">
-        <v>10.2</v>
+        <v>6.9</v>
       </c>
       <c r="M26" s="7" t="inlineStr"/>
     </row>
@@ -1542,19 +1542,19 @@
       </c>
       <c r="B27" s="7" t="inlineStr">
         <is>
-          <t>Free1ng</t>
+          <t>Yetujey</t>
         </is>
       </c>
       <c r="C27" s="7" t="inlineStr">
         <is>
-          <t>DRX</t>
+          <t>FUT Esports</t>
         </is>
       </c>
       <c r="D27" s="7" t="n">
         <v>7.5</v>
       </c>
       <c r="E27" s="7" t="n">
-        <v>6.3</v>
+        <v>7.3</v>
       </c>
       <c r="F27" s="7" t="inlineStr"/>
       <c r="H27" s="6" t="inlineStr">
@@ -1564,19 +1564,19 @@
       </c>
       <c r="I27" s="7" t="inlineStr">
         <is>
-          <t>echo</t>
+          <t>Westside</t>
         </is>
       </c>
       <c r="J27" s="7" t="inlineStr">
         <is>
-          <t>Eternal Fire</t>
+          <t>GIANTX</t>
         </is>
       </c>
       <c r="K27" s="7" t="n">
-        <v>5</v>
+        <v>7.5</v>
       </c>
       <c r="L27" s="7" t="n">
-        <v>6.9</v>
+        <v>6.4</v>
       </c>
       <c r="M27" s="7" t="inlineStr"/>
     </row>
@@ -1634,19 +1634,19 @@
       </c>
       <c r="B29" s="7" t="inlineStr">
         <is>
-          <t>xeus</t>
+          <t>Munchkin</t>
         </is>
       </c>
       <c r="C29" s="7" t="inlineStr">
         <is>
-          <t>FUT Esports</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="D29" s="7" t="n">
-        <v>10.5</v>
+        <v>7.5</v>
       </c>
       <c r="E29" s="7" t="n">
-        <v>9.800000000000001</v>
+        <v>7.2</v>
       </c>
       <c r="F29" s="7" t="inlineStr"/>
       <c r="H29" s="6" t="inlineStr">
@@ -1680,19 +1680,19 @@
       </c>
       <c r="B30" s="7" t="inlineStr">
         <is>
-          <t>Munchkin</t>
+          <t>xavi8k</t>
         </is>
       </c>
       <c r="C30" s="7" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>Global Esports</t>
         </is>
       </c>
       <c r="D30" s="7" t="n">
         <v>7.5</v>
       </c>
       <c r="E30" s="7" t="n">
-        <v>7.2</v>
+        <v>10.3</v>
       </c>
       <c r="F30" s="7" t="inlineStr"/>
       <c r="H30" s="6" t="inlineStr">
@@ -1702,19 +1702,19 @@
       </c>
       <c r="I30" s="7" t="inlineStr">
         <is>
-          <t>xeus</t>
+          <t>BuZz</t>
         </is>
       </c>
       <c r="J30" s="7" t="inlineStr">
         <is>
-          <t>FUT Esports</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="K30" s="7" t="n">
-        <v>9.5</v>
+        <v>12</v>
       </c>
       <c r="L30" s="7" t="n">
-        <v>9.800000000000001</v>
+        <v>9</v>
       </c>
       <c r="M30" s="7" t="inlineStr"/>
     </row>
@@ -1728,11 +1728,11 @@
         <v>99.5</v>
       </c>
       <c r="E31" s="9" t="n">
-        <v>100</v>
+        <v>98.8</v>
       </c>
       <c r="F31" s="5" t="inlineStr">
         <is>
-          <t>IGL: 112.0</t>
+          <t>IGL: 110.7</t>
         </is>
       </c>
       <c r="H31" s="9" t="inlineStr">
@@ -1744,11 +1744,11 @@
         <v>100</v>
       </c>
       <c r="L31" s="9" t="n">
-        <v>106</v>
+        <v>96.7</v>
       </c>
       <c r="M31" s="5" t="inlineStr">
         <is>
-          <t>IGL: 117.9</t>
+          <t>IGL: 108.6</t>
         </is>
       </c>
     </row>
@@ -1767,12 +1767,12 @@
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
         <is>
-          <t>Transfers: OUT Dos9, Kushy, Munchkin -&gt; IN supamen, cauanzin, dgzin</t>
+          <t>Transfers: [W1] Jemkin -&gt; dgzin | [C2] Dos9 -&gt; supamen | [W2] Munchkin -&gt; Ruxic</t>
         </is>
       </c>
       <c r="H34" s="5" t="inlineStr">
         <is>
-          <t>Transfers: OUT xavi8k, LewN, Kushy -&gt; IN supamen, dgzin, Verno</t>
+          <t>Transfers: [W3] BuZz -&gt; dgzin | [I2] N4RRATE -&gt; Verno | [C2] crazyguy -&gt; Erde</t>
         </is>
       </c>
     </row>
@@ -1784,25 +1784,21 @@
       </c>
       <c r="B35" s="7" t="inlineStr">
         <is>
-          <t>dgzin</t>
+          <t>LewN</t>
         </is>
       </c>
       <c r="C35" s="7" t="inlineStr">
         <is>
-          <t>Evil Geniuses</t>
+          <t>Karmine Corp</t>
         </is>
       </c>
       <c r="D35" s="7" t="n">
-        <v>11</v>
+        <v>10.5</v>
       </c>
       <c r="E35" s="7" t="n">
-        <v>11.7</v>
-      </c>
-      <c r="F35" s="8" t="inlineStr">
-        <is>
-          <t>IGL</t>
-        </is>
-      </c>
+        <v>8.800000000000001</v>
+      </c>
+      <c r="F35" s="7" t="inlineStr"/>
       <c r="H35" s="6" t="inlineStr">
         <is>
           <t>D1</t>
@@ -1810,25 +1806,21 @@
       </c>
       <c r="I35" s="7" t="inlineStr">
         <is>
-          <t>dgzin</t>
+          <t>xeus</t>
         </is>
       </c>
       <c r="J35" s="7" t="inlineStr">
         <is>
-          <t>Evil Geniuses</t>
+          <t>FUT Esports</t>
         </is>
       </c>
       <c r="K35" s="7" t="n">
-        <v>11.5</v>
+        <v>9.5</v>
       </c>
       <c r="L35" s="7" t="n">
-        <v>11.7</v>
-      </c>
-      <c r="M35" s="8" t="inlineStr">
-        <is>
-          <t>IGL</t>
-        </is>
-      </c>
+        <v>9.800000000000001</v>
+      </c>
+      <c r="M35" s="7" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
@@ -1860,19 +1852,19 @@
       </c>
       <c r="I36" s="7" t="inlineStr">
         <is>
-          <t>Lar0k</t>
+          <t>LewN</t>
         </is>
       </c>
       <c r="J36" s="7" t="inlineStr">
         <is>
-          <t>BBL Esports</t>
+          <t>Karmine Corp</t>
         </is>
       </c>
       <c r="K36" s="7" t="n">
-        <v>9.5</v>
+        <v>11.5</v>
       </c>
       <c r="L36" s="7" t="n">
-        <v>10.9</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="M36" s="7" t="inlineStr"/>
     </row>
@@ -1884,19 +1876,19 @@
       </c>
       <c r="B37" s="7" t="inlineStr">
         <is>
-          <t>Rosé</t>
+          <t>Kushy</t>
         </is>
       </c>
       <c r="C37" s="7" t="inlineStr">
         <is>
-          <t>BBL Esports</t>
+          <t>Rex Regum Qeon</t>
         </is>
       </c>
       <c r="D37" s="7" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E37" s="7" t="n">
-        <v>7.9</v>
+        <v>6.9</v>
       </c>
       <c r="F37" s="7" t="inlineStr"/>
       <c r="H37" s="6" t="inlineStr">
@@ -1906,19 +1898,19 @@
       </c>
       <c r="I37" s="7" t="inlineStr">
         <is>
-          <t>Verno</t>
+          <t>Kushy</t>
         </is>
       </c>
       <c r="J37" s="7" t="inlineStr">
         <is>
-          <t>MIBR</t>
+          <t>Rex Regum Qeon</t>
         </is>
       </c>
       <c r="K37" s="7" t="n">
         <v>8.5</v>
       </c>
       <c r="L37" s="7" t="n">
-        <v>8</v>
+        <v>6.9</v>
       </c>
       <c r="M37" s="7" t="inlineStr"/>
     </row>
@@ -1930,19 +1922,19 @@
       </c>
       <c r="B38" s="7" t="inlineStr">
         <is>
-          <t>cauanzin</t>
+          <t>Rosé</t>
         </is>
       </c>
       <c r="C38" s="7" t="inlineStr">
         <is>
-          <t>LOUD</t>
+          <t>BBL Esports</t>
         </is>
       </c>
       <c r="D38" s="7" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E38" s="7" t="n">
-        <v>7</v>
+        <v>7.9</v>
       </c>
       <c r="F38" s="7" t="inlineStr"/>
       <c r="H38" s="6" t="inlineStr">
@@ -1952,19 +1944,19 @@
       </c>
       <c r="I38" s="7" t="inlineStr">
         <is>
-          <t>cloud</t>
+          <t>Verno</t>
         </is>
       </c>
       <c r="J38" s="7" t="inlineStr">
         <is>
-          <t>GIANTX</t>
+          <t>MIBR</t>
         </is>
       </c>
       <c r="K38" s="7" t="n">
-        <v>7</v>
+        <v>8.5</v>
       </c>
       <c r="L38" s="7" t="n">
-        <v>6.5</v>
+        <v>8</v>
       </c>
       <c r="M38" s="7" t="inlineStr"/>
     </row>
@@ -1976,19 +1968,19 @@
       </c>
       <c r="B39" s="7" t="inlineStr">
         <is>
-          <t>supamen</t>
+          <t>Veqaj</t>
         </is>
       </c>
       <c r="C39" s="7" t="inlineStr">
         <is>
-          <t>Evil Geniuses</t>
+          <t>FNATIC</t>
         </is>
       </c>
       <c r="D39" s="7" t="n">
-        <v>6.5</v>
+        <v>10.5</v>
       </c>
       <c r="E39" s="7" t="n">
-        <v>8.199999999999999</v>
+        <v>9.9</v>
       </c>
       <c r="F39" s="7" t="inlineStr"/>
       <c r="H39" s="6" t="inlineStr">
@@ -2022,19 +2014,19 @@
       </c>
       <c r="B40" s="7" t="inlineStr">
         <is>
-          <t>xavi8k</t>
+          <t>supamen</t>
         </is>
       </c>
       <c r="C40" s="7" t="inlineStr">
         <is>
-          <t>Global Esports</t>
+          <t>Evil Geniuses</t>
         </is>
       </c>
       <c r="D40" s="7" t="n">
-        <v>7.5</v>
+        <v>6.5</v>
       </c>
       <c r="E40" s="7" t="n">
-        <v>7.6</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="F40" s="7" t="inlineStr"/>
       <c r="H40" s="6" t="inlineStr">
@@ -2044,19 +2036,19 @@
       </c>
       <c r="I40" s="7" t="inlineStr">
         <is>
-          <t>supamen</t>
+          <t>Erde</t>
         </is>
       </c>
       <c r="J40" s="7" t="inlineStr">
         <is>
-          <t>Evil Geniuses</t>
+          <t>LOUD</t>
         </is>
       </c>
       <c r="K40" s="7" t="n">
-        <v>8.5</v>
+        <v>6.5</v>
       </c>
       <c r="L40" s="7" t="n">
-        <v>8.199999999999999</v>
+        <v>6.9</v>
       </c>
       <c r="M40" s="7" t="inlineStr"/>
     </row>
@@ -2090,19 +2082,19 @@
       </c>
       <c r="I41" s="7" t="inlineStr">
         <is>
-          <t>skuba</t>
+          <t>caedye</t>
         </is>
       </c>
       <c r="J41" s="7" t="inlineStr">
         <is>
-          <t>NRG Esports</t>
+          <t>Detonation FocusMe</t>
         </is>
       </c>
       <c r="K41" s="7" t="n">
-        <v>13</v>
+        <v>8.5</v>
       </c>
       <c r="L41" s="7" t="n">
-        <v>8.9</v>
+        <v>7.9</v>
       </c>
       <c r="M41" s="7" t="inlineStr"/>
     </row>
@@ -2136,19 +2128,19 @@
       </c>
       <c r="I42" s="7" t="inlineStr">
         <is>
-          <t>echo</t>
+          <t>Westside</t>
         </is>
       </c>
       <c r="J42" s="7" t="inlineStr">
         <is>
-          <t>Eternal Fire</t>
+          <t>GIANTX</t>
         </is>
       </c>
       <c r="K42" s="7" t="n">
-        <v>5</v>
+        <v>7.5</v>
       </c>
       <c r="L42" s="7" t="n">
-        <v>6.9</v>
+        <v>5.6</v>
       </c>
       <c r="M42" s="7" t="inlineStr"/>
     </row>
@@ -2160,21 +2152,25 @@
       </c>
       <c r="B43" s="7" t="inlineStr">
         <is>
-          <t>xeus</t>
+          <t>dgzin</t>
         </is>
       </c>
       <c r="C43" s="7" t="inlineStr">
         <is>
-          <t>FUT Esports</t>
+          <t>Evil Geniuses</t>
         </is>
       </c>
       <c r="D43" s="7" t="n">
-        <v>10.5</v>
+        <v>11</v>
       </c>
       <c r="E43" s="7" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="F43" s="7" t="inlineStr"/>
+        <v>11.7</v>
+      </c>
+      <c r="F43" s="8" t="inlineStr">
+        <is>
+          <t>IGL</t>
+        </is>
+      </c>
       <c r="H43" s="6" t="inlineStr">
         <is>
           <t>W1</t>
@@ -2182,7 +2178,7 @@
       </c>
       <c r="I43" s="7" t="inlineStr">
         <is>
-          <t>Lovers rock</t>
+          <t>Lar0k</t>
         </is>
       </c>
       <c r="J43" s="7" t="inlineStr">
@@ -2191,10 +2187,10 @@
         </is>
       </c>
       <c r="K43" s="7" t="n">
-        <v>9</v>
+        <v>9.5</v>
       </c>
       <c r="L43" s="7" t="n">
-        <v>10.7</v>
+        <v>10.9</v>
       </c>
       <c r="M43" s="7" t="inlineStr"/>
     </row>
@@ -2206,19 +2202,19 @@
       </c>
       <c r="B44" s="7" t="inlineStr">
         <is>
-          <t>Jemkin</t>
+          <t>Ruxic</t>
         </is>
       </c>
       <c r="C44" s="7" t="inlineStr">
         <is>
-          <t>Rex Regum Qeon</t>
+          <t>Natus Vincere</t>
         </is>
       </c>
       <c r="D44" s="7" t="n">
-        <v>13.5</v>
+        <v>11.5</v>
       </c>
       <c r="E44" s="7" t="n">
-        <v>9</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="F44" s="7" t="inlineStr"/>
       <c r="H44" s="6" t="inlineStr">
@@ -2228,19 +2224,19 @@
       </c>
       <c r="I44" s="7" t="inlineStr">
         <is>
-          <t>xeus</t>
+          <t>Lovers rock</t>
         </is>
       </c>
       <c r="J44" s="7" t="inlineStr">
         <is>
-          <t>FUT Esports</t>
+          <t>BBL Esports</t>
         </is>
       </c>
       <c r="K44" s="7" t="n">
-        <v>9.5</v>
+        <v>9</v>
       </c>
       <c r="L44" s="7" t="n">
-        <v>9.800000000000001</v>
+        <v>10.7</v>
       </c>
       <c r="M44" s="7" t="inlineStr"/>
     </row>
@@ -2252,19 +2248,19 @@
       </c>
       <c r="B45" s="7" t="inlineStr">
         <is>
-          <t>LewN</t>
+          <t>xavi8k</t>
         </is>
       </c>
       <c r="C45" s="7" t="inlineStr">
         <is>
-          <t>Karmine Corp</t>
+          <t>Global Esports</t>
         </is>
       </c>
       <c r="D45" s="7" t="n">
-        <v>10.5</v>
+        <v>7.5</v>
       </c>
       <c r="E45" s="7" t="n">
-        <v>8.800000000000001</v>
+        <v>7.6</v>
       </c>
       <c r="F45" s="7" t="inlineStr"/>
       <c r="H45" s="6" t="inlineStr">
@@ -2274,21 +2270,25 @@
       </c>
       <c r="I45" s="7" t="inlineStr">
         <is>
-          <t>Autumn</t>
+          <t>dgzin</t>
         </is>
       </c>
       <c r="J45" s="7" t="inlineStr">
         <is>
-          <t>Global Esports</t>
+          <t>Evil Geniuses</t>
         </is>
       </c>
       <c r="K45" s="7" t="n">
-        <v>8.5</v>
+        <v>11.5</v>
       </c>
       <c r="L45" s="7" t="n">
-        <v>8.199999999999999</v>
-      </c>
-      <c r="M45" s="7" t="inlineStr"/>
+        <v>11.7</v>
+      </c>
+      <c r="M45" s="8" t="inlineStr">
+        <is>
+          <t>IGL</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="9" t="inlineStr">
@@ -2300,11 +2300,11 @@
         <v>99.5</v>
       </c>
       <c r="E46" s="9" t="n">
-        <v>96.90000000000001</v>
+        <v>97.5</v>
       </c>
       <c r="F46" s="5" t="inlineStr">
         <is>
-          <t>IGL: 108.6</t>
+          <t>IGL: 109.2</t>
         </is>
       </c>
       <c r="H46" s="9" t="inlineStr">
@@ -2313,14 +2313,14 @@
         </is>
       </c>
       <c r="J46" s="9" t="n">
-        <v>99.5</v>
+        <v>100</v>
       </c>
       <c r="L46" s="9" t="n">
-        <v>99.8</v>
+        <v>97.2</v>
       </c>
       <c r="M46" s="5" t="inlineStr">
         <is>
-          <t>IGL: 111.4</t>
+          <t>IGL: 108.9</t>
         </is>
       </c>
     </row>
@@ -2339,12 +2339,12 @@
     <row r="49">
       <c r="A49" s="5" t="inlineStr">
         <is>
-          <t>Transfers: OUT Jemkin, supamen, Free1ng -&gt; IN jawgemo, Saadhak, Less</t>
+          <t>Transfers: [S1] Free1ng -&gt; Zellsis | [W2] Ruxic -&gt; jawgemo | [S1] Zellsis -&gt; echo</t>
         </is>
       </c>
       <c r="H49" s="5" t="inlineStr">
         <is>
-          <t>Transfers: OUT dgzin, supamen, cloud -&gt; IN BABYBAY, Saadhak, eeiu</t>
+          <t>Transfers: [S2] Westside -&gt; echo | [S1] caedye -&gt; Less | [W3] dgzin -&gt; BABYBAY</t>
         </is>
       </c>
     </row>
@@ -2356,25 +2356,21 @@
       </c>
       <c r="B50" s="7" t="inlineStr">
         <is>
-          <t>jawgemo</t>
+          <t>LewN</t>
         </is>
       </c>
       <c r="C50" s="7" t="inlineStr">
         <is>
-          <t>G2 Esports</t>
+          <t>Karmine Corp</t>
         </is>
       </c>
       <c r="D50" s="7" t="n">
-        <v>13.5</v>
+        <v>10.5</v>
       </c>
       <c r="E50" s="7" t="n">
-        <v>11.1</v>
-      </c>
-      <c r="F50" s="8" t="inlineStr">
-        <is>
-          <t>IGL</t>
-        </is>
-      </c>
+        <v>10.4</v>
+      </c>
+      <c r="F50" s="7" t="inlineStr"/>
       <c r="H50" s="6" t="inlineStr">
         <is>
           <t>D1</t>
@@ -2382,25 +2378,21 @@
       </c>
       <c r="I50" s="7" t="inlineStr">
         <is>
-          <t>BABYBAY</t>
+          <t>xeus</t>
         </is>
       </c>
       <c r="J50" s="7" t="inlineStr">
         <is>
-          <t>G2 Esports</t>
+          <t>FUT Esports</t>
         </is>
       </c>
       <c r="K50" s="7" t="n">
-        <v>12</v>
+        <v>9.5</v>
       </c>
       <c r="L50" s="7" t="n">
-        <v>10.1</v>
-      </c>
-      <c r="M50" s="8" t="inlineStr">
-        <is>
-          <t>IGL</t>
-        </is>
-      </c>
+        <v>9.800000000000001</v>
+      </c>
+      <c r="M50" s="7" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="6" t="inlineStr">
@@ -2410,19 +2402,19 @@
       </c>
       <c r="B51" s="7" t="inlineStr">
         <is>
-          <t>LewN</t>
+          <t>Lar0k</t>
         </is>
       </c>
       <c r="C51" s="7" t="inlineStr">
         <is>
-          <t>Karmine Corp</t>
+          <t>BBL Esports</t>
         </is>
       </c>
       <c r="D51" s="7" t="n">
-        <v>10.5</v>
+        <v>12</v>
       </c>
       <c r="E51" s="7" t="n">
-        <v>10.4</v>
+        <v>9.5</v>
       </c>
       <c r="F51" s="7" t="inlineStr"/>
       <c r="H51" s="6" t="inlineStr">
@@ -2432,21 +2424,25 @@
       </c>
       <c r="I51" s="7" t="inlineStr">
         <is>
-          <t>xeus</t>
+          <t>LewN</t>
         </is>
       </c>
       <c r="J51" s="7" t="inlineStr">
         <is>
-          <t>FUT Esports</t>
+          <t>Karmine Corp</t>
         </is>
       </c>
       <c r="K51" s="7" t="n">
-        <v>9.5</v>
+        <v>11.5</v>
       </c>
       <c r="L51" s="7" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="M51" s="7" t="inlineStr"/>
+        <v>10.4</v>
+      </c>
+      <c r="M51" s="8" t="inlineStr">
+        <is>
+          <t>IGL</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="6" t="inlineStr">
@@ -2456,16 +2452,16 @@
       </c>
       <c r="B52" s="7" t="inlineStr">
         <is>
-          <t>Rosé</t>
+          <t>Kushy</t>
         </is>
       </c>
       <c r="C52" s="7" t="inlineStr">
         <is>
-          <t>BBL Esports</t>
+          <t>Rex Regum Qeon</t>
         </is>
       </c>
       <c r="D52" s="7" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E52" s="7" t="n">
         <v>6.9</v>
@@ -2478,19 +2474,19 @@
       </c>
       <c r="I52" s="7" t="inlineStr">
         <is>
-          <t>eeiu</t>
+          <t>Kushy</t>
         </is>
       </c>
       <c r="J52" s="7" t="inlineStr">
         <is>
-          <t>FURIA</t>
+          <t>Rex Regum Qeon</t>
         </is>
       </c>
       <c r="K52" s="7" t="n">
-        <v>9</v>
+        <v>8.5</v>
       </c>
       <c r="L52" s="7" t="n">
-        <v>7.3</v>
+        <v>6.9</v>
       </c>
       <c r="M52" s="7" t="inlineStr"/>
     </row>
@@ -2502,19 +2498,19 @@
       </c>
       <c r="B53" s="7" t="inlineStr">
         <is>
-          <t>cauanzin</t>
+          <t>Rosé</t>
         </is>
       </c>
       <c r="C53" s="7" t="inlineStr">
         <is>
-          <t>LOUD</t>
+          <t>BBL Esports</t>
         </is>
       </c>
       <c r="D53" s="7" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E53" s="7" t="n">
-        <v>5.9</v>
+        <v>6.9</v>
       </c>
       <c r="F53" s="7" t="inlineStr"/>
       <c r="H53" s="6" t="inlineStr">
@@ -2548,19 +2544,19 @@
       </c>
       <c r="B54" s="7" t="inlineStr">
         <is>
-          <t>xavi8k</t>
+          <t>Veqaj</t>
         </is>
       </c>
       <c r="C54" s="7" t="inlineStr">
         <is>
-          <t>Global Esports</t>
+          <t>FNATIC</t>
         </is>
       </c>
       <c r="D54" s="7" t="n">
-        <v>7.5</v>
+        <v>10.5</v>
       </c>
       <c r="E54" s="7" t="n">
-        <v>7.6</v>
+        <v>9.9</v>
       </c>
       <c r="F54" s="7" t="inlineStr"/>
       <c r="H54" s="6" t="inlineStr">
@@ -2594,19 +2590,19 @@
       </c>
       <c r="B55" s="7" t="inlineStr">
         <is>
-          <t>Saadhak</t>
+          <t>supamen</t>
         </is>
       </c>
       <c r="C55" s="7" t="inlineStr">
         <is>
-          <t>KRU Esports</t>
+          <t>Evil Geniuses</t>
         </is>
       </c>
       <c r="D55" s="7" t="n">
-        <v>6</v>
+        <v>6.5</v>
       </c>
       <c r="E55" s="7" t="n">
-        <v>5.9</v>
+        <v>6.1</v>
       </c>
       <c r="F55" s="7" t="inlineStr"/>
       <c r="H55" s="6" t="inlineStr">
@@ -2616,16 +2612,16 @@
       </c>
       <c r="I55" s="7" t="inlineStr">
         <is>
-          <t>Saadhak</t>
+          <t>Erde</t>
         </is>
       </c>
       <c r="J55" s="7" t="inlineStr">
         <is>
-          <t>KRU Esports</t>
+          <t>LOUD</t>
         </is>
       </c>
       <c r="K55" s="7" t="n">
-        <v>6</v>
+        <v>6.5</v>
       </c>
       <c r="L55" s="7" t="n">
         <v>5.9</v>
@@ -2640,19 +2636,19 @@
       </c>
       <c r="B56" s="7" t="inlineStr">
         <is>
-          <t>Less</t>
+          <t>echo</t>
         </is>
       </c>
       <c r="C56" s="7" t="inlineStr">
         <is>
-          <t>KRU Esports</t>
+          <t>Eternal Fire</t>
         </is>
       </c>
       <c r="D56" s="7" t="n">
-        <v>8.5</v>
+        <v>6</v>
       </c>
       <c r="E56" s="7" t="n">
-        <v>8.5</v>
+        <v>7.9</v>
       </c>
       <c r="F56" s="7" t="inlineStr"/>
       <c r="H56" s="6" t="inlineStr">
@@ -2662,19 +2658,19 @@
       </c>
       <c r="I56" s="7" t="inlineStr">
         <is>
-          <t>skuba</t>
+          <t>Less</t>
         </is>
       </c>
       <c r="J56" s="7" t="inlineStr">
         <is>
-          <t>NRG Esports</t>
+          <t>KRU Esports</t>
         </is>
       </c>
       <c r="K56" s="7" t="n">
-        <v>13</v>
+        <v>10.5</v>
       </c>
       <c r="L56" s="7" t="n">
-        <v>8.9</v>
+        <v>8.5</v>
       </c>
       <c r="M56" s="7" t="inlineStr"/>
     </row>
@@ -2732,19 +2728,19 @@
       </c>
       <c r="B58" s="7" t="inlineStr">
         <is>
-          <t>xeus</t>
+          <t>dgzin</t>
         </is>
       </c>
       <c r="C58" s="7" t="inlineStr">
         <is>
-          <t>FUT Esports</t>
+          <t>Evil Geniuses</t>
         </is>
       </c>
       <c r="D58" s="7" t="n">
-        <v>10.5</v>
+        <v>11</v>
       </c>
       <c r="E58" s="7" t="n">
-        <v>9.800000000000001</v>
+        <v>8.6</v>
       </c>
       <c r="F58" s="7" t="inlineStr"/>
       <c r="H58" s="6" t="inlineStr">
@@ -2778,21 +2774,25 @@
       </c>
       <c r="B59" s="7" t="inlineStr">
         <is>
-          <t>Lar0k</t>
+          <t>jawgemo</t>
         </is>
       </c>
       <c r="C59" s="7" t="inlineStr">
         <is>
-          <t>BBL Esports</t>
+          <t>G2 Esports</t>
         </is>
       </c>
       <c r="D59" s="7" t="n">
-        <v>12</v>
+        <v>13.5</v>
       </c>
       <c r="E59" s="7" t="n">
-        <v>9.5</v>
-      </c>
-      <c r="F59" s="7" t="inlineStr"/>
+        <v>11.1</v>
+      </c>
+      <c r="F59" s="8" t="inlineStr">
+        <is>
+          <t>IGL</t>
+        </is>
+      </c>
       <c r="H59" s="6" t="inlineStr">
         <is>
           <t>W2</t>
@@ -2824,19 +2824,19 @@
       </c>
       <c r="B60" s="7" t="inlineStr">
         <is>
-          <t>dgzin</t>
+          <t>xavi8k</t>
         </is>
       </c>
       <c r="C60" s="7" t="inlineStr">
         <is>
-          <t>Evil Geniuses</t>
+          <t>Global Esports</t>
         </is>
       </c>
       <c r="D60" s="7" t="n">
-        <v>11</v>
+        <v>7.5</v>
       </c>
       <c r="E60" s="7" t="n">
-        <v>8.6</v>
+        <v>7.6</v>
       </c>
       <c r="F60" s="7" t="inlineStr"/>
       <c r="H60" s="6" t="inlineStr">
@@ -2846,19 +2846,19 @@
       </c>
       <c r="I60" s="7" t="inlineStr">
         <is>
-          <t>Autumn</t>
+          <t>BABYBAY</t>
         </is>
       </c>
       <c r="J60" s="7" t="inlineStr">
         <is>
-          <t>Global Esports</t>
+          <t>G2 Esports</t>
         </is>
       </c>
       <c r="K60" s="7" t="n">
-        <v>8.5</v>
+        <v>12</v>
       </c>
       <c r="L60" s="7" t="n">
-        <v>8.199999999999999</v>
+        <v>10.1</v>
       </c>
       <c r="M60" s="7" t="inlineStr"/>
     </row>
@@ -2872,11 +2872,11 @@
         <v>100</v>
       </c>
       <c r="E61" s="9" t="n">
-        <v>91.7</v>
+        <v>92.3</v>
       </c>
       <c r="F61" s="5" t="inlineStr">
         <is>
-          <t>IGL: 102.8</t>
+          <t>IGL: 103.4</t>
         </is>
       </c>
       <c r="H61" s="9" t="inlineStr">
@@ -2885,14 +2885,14 @@
         </is>
       </c>
       <c r="J61" s="9" t="n">
-        <v>99.5</v>
+        <v>100</v>
       </c>
       <c r="L61" s="9" t="n">
-        <v>93.8</v>
+        <v>95.3</v>
       </c>
       <c r="M61" s="5" t="inlineStr">
         <is>
-          <t>IGL: 104.0</t>
+          <t>IGL: 105.7</t>
         </is>
       </c>
     </row>
@@ -2911,12 +2911,12 @@
     <row r="64">
       <c r="A64" s="5" t="inlineStr">
         <is>
-          <t>Transfers: OUT Lar0k, Saadhak, Rosé -&gt; IN JohnQT, v1c, JonahP</t>
+          <t>Transfers: [C1] Veqaj -&gt; v1c | [S2] Yetujey -&gt; skuba | [I2] Rosé -&gt; Xeppaa</t>
         </is>
       </c>
       <c r="H64" s="5" t="inlineStr">
         <is>
-          <t>Transfers: OUT Saadhak, BABYBAY, eeiu -&gt; IN Erde, OXY, Xeppaa</t>
+          <t>Transfers: [I1] Kushy -&gt; Xeppaa | [W3] BABYBAY -&gt; OXY | [W2] Lovers rock -&gt; Neon</t>
         </is>
       </c>
     </row>
@@ -2954,25 +2954,21 @@
       </c>
       <c r="I65" s="7" t="inlineStr">
         <is>
-          <t>OXY</t>
+          <t>xeus</t>
         </is>
       </c>
       <c r="J65" s="7" t="inlineStr">
         <is>
-          <t>Cloud9</t>
+          <t>FUT Esports</t>
         </is>
       </c>
       <c r="K65" s="7" t="n">
-        <v>12</v>
+        <v>9.5</v>
       </c>
       <c r="L65" s="7" t="n">
-        <v>10.7</v>
-      </c>
-      <c r="M65" s="8" t="inlineStr">
-        <is>
-          <t>IGL</t>
-        </is>
-      </c>
+        <v>8.4</v>
+      </c>
+      <c r="M65" s="7" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" s="6" t="inlineStr">
@@ -2982,19 +2978,19 @@
       </c>
       <c r="B66" s="7" t="inlineStr">
         <is>
-          <t>jawgemo</t>
+          <t>Lar0k</t>
         </is>
       </c>
       <c r="C66" s="7" t="inlineStr">
         <is>
-          <t>G2 Esports</t>
+          <t>BBL Esports</t>
         </is>
       </c>
       <c r="D66" s="7" t="n">
-        <v>13.5</v>
+        <v>12</v>
       </c>
       <c r="E66" s="7" t="n">
-        <v>9.699999999999999</v>
+        <v>8.1</v>
       </c>
       <c r="F66" s="7" t="inlineStr"/>
       <c r="H66" s="6" t="inlineStr">
@@ -3004,19 +3000,19 @@
       </c>
       <c r="I66" s="7" t="inlineStr">
         <is>
-          <t>xeus</t>
+          <t>LewN</t>
         </is>
       </c>
       <c r="J66" s="7" t="inlineStr">
         <is>
-          <t>FUT Esports</t>
+          <t>Karmine Corp</t>
         </is>
       </c>
       <c r="K66" s="7" t="n">
-        <v>9.5</v>
+        <v>11.5</v>
       </c>
       <c r="L66" s="7" t="n">
-        <v>8.4</v>
+        <v>10.4</v>
       </c>
       <c r="M66" s="7" t="inlineStr"/>
     </row>
@@ -3028,19 +3024,19 @@
       </c>
       <c r="B67" s="7" t="inlineStr">
         <is>
-          <t>JonahP</t>
+          <t>Kushy</t>
         </is>
       </c>
       <c r="C67" s="7" t="inlineStr">
         <is>
-          <t>Sentinels</t>
+          <t>Rex Regum Qeon</t>
         </is>
       </c>
       <c r="D67" s="7" t="n">
         <v>8</v>
       </c>
       <c r="E67" s="7" t="n">
-        <v>8.4</v>
+        <v>6.9</v>
       </c>
       <c r="F67" s="7" t="inlineStr"/>
       <c r="H67" s="6" t="inlineStr">
@@ -3074,19 +3070,19 @@
       </c>
       <c r="B68" s="7" t="inlineStr">
         <is>
-          <t>cauanzin</t>
+          <t>Xeppaa</t>
         </is>
       </c>
       <c r="C68" s="7" t="inlineStr">
         <is>
-          <t>LOUD</t>
+          <t>Cloud9</t>
         </is>
       </c>
       <c r="D68" s="7" t="n">
-        <v>6</v>
+        <v>7.5</v>
       </c>
       <c r="E68" s="7" t="n">
-        <v>7</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="F68" s="7" t="inlineStr"/>
       <c r="H68" s="6" t="inlineStr">
@@ -3166,19 +3162,19 @@
       </c>
       <c r="B70" s="7" t="inlineStr">
         <is>
-          <t>JohnQT</t>
+          <t>supamen</t>
         </is>
       </c>
       <c r="C70" s="7" t="inlineStr">
         <is>
-          <t>Sentinels</t>
+          <t>Evil Geniuses</t>
         </is>
       </c>
       <c r="D70" s="7" t="n">
-        <v>9</v>
+        <v>6.5</v>
       </c>
       <c r="E70" s="7" t="n">
-        <v>9</v>
+        <v>6.1</v>
       </c>
       <c r="F70" s="7" t="inlineStr"/>
       <c r="H70" s="6" t="inlineStr">
@@ -3212,19 +3208,19 @@
       </c>
       <c r="B71" s="7" t="inlineStr">
         <is>
-          <t>Less</t>
+          <t>echo</t>
         </is>
       </c>
       <c r="C71" s="7" t="inlineStr">
         <is>
-          <t>KRU Esports</t>
+          <t>Eternal Fire</t>
         </is>
       </c>
       <c r="D71" s="7" t="n">
-        <v>8.5</v>
+        <v>6</v>
       </c>
       <c r="E71" s="7" t="n">
-        <v>7.4</v>
+        <v>7.9</v>
       </c>
       <c r="F71" s="7" t="inlineStr"/>
       <c r="H71" s="6" t="inlineStr">
@@ -3234,19 +3230,19 @@
       </c>
       <c r="I71" s="7" t="inlineStr">
         <is>
-          <t>skuba</t>
+          <t>Less</t>
         </is>
       </c>
       <c r="J71" s="7" t="inlineStr">
         <is>
-          <t>NRG Esports</t>
+          <t>KRU Esports</t>
         </is>
       </c>
       <c r="K71" s="7" t="n">
-        <v>13</v>
+        <v>10.5</v>
       </c>
       <c r="L71" s="7" t="n">
-        <v>8.9</v>
+        <v>7.4</v>
       </c>
       <c r="M71" s="7" t="inlineStr"/>
     </row>
@@ -3258,19 +3254,19 @@
       </c>
       <c r="B72" s="7" t="inlineStr">
         <is>
-          <t>Yetujey</t>
+          <t>skuba</t>
         </is>
       </c>
       <c r="C72" s="7" t="inlineStr">
         <is>
-          <t>FUT Esports</t>
+          <t>NRG Esports</t>
         </is>
       </c>
       <c r="D72" s="7" t="n">
-        <v>7.5</v>
+        <v>9.5</v>
       </c>
       <c r="E72" s="7" t="n">
-        <v>6.2</v>
+        <v>8.9</v>
       </c>
       <c r="F72" s="7" t="inlineStr"/>
       <c r="H72" s="6" t="inlineStr">
@@ -3326,19 +3322,19 @@
       </c>
       <c r="I73" s="7" t="inlineStr">
         <is>
-          <t>Autumn</t>
+          <t>Lar0k</t>
         </is>
       </c>
       <c r="J73" s="7" t="inlineStr">
         <is>
-          <t>Global Esports</t>
+          <t>BBL Esports</t>
         </is>
       </c>
       <c r="K73" s="7" t="n">
-        <v>8.5</v>
+        <v>9.5</v>
       </c>
       <c r="L73" s="7" t="n">
-        <v>8.199999999999999</v>
+        <v>8.1</v>
       </c>
       <c r="M73" s="7" t="inlineStr"/>
     </row>
@@ -3350,19 +3346,19 @@
       </c>
       <c r="B74" s="7" t="inlineStr">
         <is>
-          <t>xeus</t>
+          <t>jawgemo</t>
         </is>
       </c>
       <c r="C74" s="7" t="inlineStr">
         <is>
-          <t>FUT Esports</t>
+          <t>G2 Esports</t>
         </is>
       </c>
       <c r="D74" s="7" t="n">
-        <v>10.5</v>
+        <v>13.5</v>
       </c>
       <c r="E74" s="7" t="n">
-        <v>8.4</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="F74" s="7" t="inlineStr"/>
       <c r="H74" s="6" t="inlineStr">
@@ -3372,19 +3368,19 @@
       </c>
       <c r="I74" s="7" t="inlineStr">
         <is>
-          <t>Lar0k</t>
+          <t>Neon</t>
         </is>
       </c>
       <c r="J74" s="7" t="inlineStr">
         <is>
-          <t>BBL Esports</t>
+          <t>LEVIATAN</t>
         </is>
       </c>
       <c r="K74" s="7" t="n">
-        <v>9.5</v>
+        <v>8.5</v>
       </c>
       <c r="L74" s="7" t="n">
-        <v>8.1</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="M74" s="7" t="inlineStr"/>
     </row>
@@ -3418,21 +3414,25 @@
       </c>
       <c r="I75" s="7" t="inlineStr">
         <is>
-          <t>Lovers rock</t>
+          <t>OXY</t>
         </is>
       </c>
       <c r="J75" s="7" t="inlineStr">
         <is>
-          <t>BBL Esports</t>
+          <t>Cloud9</t>
         </is>
       </c>
       <c r="K75" s="7" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="L75" s="7" t="n">
-        <v>7.9</v>
-      </c>
-      <c r="M75" s="7" t="inlineStr"/>
+        <v>10.7</v>
+      </c>
+      <c r="M75" s="8" t="inlineStr">
+        <is>
+          <t>IGL</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="9" t="inlineStr">
@@ -3444,11 +3444,11 @@
         <v>100</v>
       </c>
       <c r="E76" s="9" t="n">
-        <v>92.09999999999999</v>
+        <v>91.90000000000001</v>
       </c>
       <c r="F76" s="5" t="inlineStr">
         <is>
-          <t>IGL: 102.5</t>
+          <t>IGL: 102.3</t>
         </is>
       </c>
       <c r="H76" s="9" t="inlineStr">
@@ -3460,11 +3460,11 @@
         <v>99.5</v>
       </c>
       <c r="L76" s="9" t="n">
-        <v>90.8</v>
+        <v>92.40000000000001</v>
       </c>
       <c r="M76" s="5" t="inlineStr">
         <is>
-          <t>IGL: 101.5</t>
+          <t>IGL: 103.1</t>
         </is>
       </c>
     </row>
@@ -3483,12 +3483,12 @@
     <row r="79">
       <c r="A79" s="5" t="inlineStr">
         <is>
-          <t>Transfers: OUT xavi8k, LewN, xeus -&gt; IN supamen, Cryocells, Neon</t>
+          <t>Transfers: [I1] Kushy -&gt; cauanzin | [D2] Lar0k -&gt; Sato | [D1] LewN -&gt; Neon</t>
         </is>
       </c>
       <c r="H79" s="5" t="inlineStr">
         <is>
-          <t>Transfers: OUT Lovers rock, Lar0k, xeus -&gt; IN Neon, Timotino, Sato</t>
+          <t>Transfers: [W1] Lar0k -&gt; Timotino | [D1] xeus -&gt; Sato | [D2] LewN -&gt; dgzin</t>
         </is>
       </c>
     </row>
@@ -3500,16 +3500,16 @@
       </c>
       <c r="B80" s="7" t="inlineStr">
         <is>
-          <t>dgzin</t>
+          <t>Neon</t>
         </is>
       </c>
       <c r="C80" s="7" t="inlineStr">
         <is>
-          <t>Evil Geniuses</t>
+          <t>LEVIATAN</t>
         </is>
       </c>
       <c r="D80" s="7" t="n">
-        <v>11</v>
+        <v>11.5</v>
       </c>
       <c r="E80" s="7" t="n">
         <v>10.1</v>
@@ -3522,7 +3522,7 @@
       </c>
       <c r="I80" s="7" t="inlineStr">
         <is>
-          <t>Neon</t>
+          <t>Sato</t>
         </is>
       </c>
       <c r="J80" s="7" t="inlineStr">
@@ -3531,16 +3531,12 @@
         </is>
       </c>
       <c r="K80" s="7" t="n">
-        <v>8.5</v>
+        <v>10.5</v>
       </c>
       <c r="L80" s="7" t="n">
-        <v>10.1</v>
-      </c>
-      <c r="M80" s="8" t="inlineStr">
-        <is>
-          <t>IGL</t>
-        </is>
-      </c>
+        <v>9.800000000000001</v>
+      </c>
+      <c r="M80" s="7" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" s="6" t="inlineStr">
@@ -3550,7 +3546,7 @@
       </c>
       <c r="B81" s="7" t="inlineStr">
         <is>
-          <t>Neon</t>
+          <t>Sato</t>
         </is>
       </c>
       <c r="C81" s="7" t="inlineStr">
@@ -3559,10 +3555,10 @@
         </is>
       </c>
       <c r="D81" s="7" t="n">
-        <v>11.5</v>
+        <v>13</v>
       </c>
       <c r="E81" s="7" t="n">
-        <v>10.1</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="F81" s="7" t="inlineStr"/>
       <c r="H81" s="6" t="inlineStr">
@@ -3572,21 +3568,25 @@
       </c>
       <c r="I81" s="7" t="inlineStr">
         <is>
-          <t>Sato</t>
+          <t>dgzin</t>
         </is>
       </c>
       <c r="J81" s="7" t="inlineStr">
         <is>
-          <t>LEVIATAN</t>
+          <t>Evil Geniuses</t>
         </is>
       </c>
       <c r="K81" s="7" t="n">
-        <v>10.5</v>
+        <v>11.5</v>
       </c>
       <c r="L81" s="7" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="M81" s="7" t="inlineStr"/>
+        <v>10.1</v>
+      </c>
+      <c r="M81" s="8" t="inlineStr">
+        <is>
+          <t>IGL</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="6" t="inlineStr">
@@ -3618,19 +3618,19 @@
       </c>
       <c r="I82" s="7" t="inlineStr">
         <is>
-          <t>Verno</t>
+          <t>Xeppaa</t>
         </is>
       </c>
       <c r="J82" s="7" t="inlineStr">
         <is>
-          <t>MIBR</t>
+          <t>Cloud9</t>
         </is>
       </c>
       <c r="K82" s="7" t="n">
         <v>8.5</v>
       </c>
       <c r="L82" s="7" t="n">
-        <v>6.9</v>
+        <v>6.2</v>
       </c>
       <c r="M82" s="7" t="inlineStr"/>
     </row>
@@ -3642,16 +3642,16 @@
       </c>
       <c r="B83" s="7" t="inlineStr">
         <is>
-          <t>JonahP</t>
+          <t>Xeppaa</t>
         </is>
       </c>
       <c r="C83" s="7" t="inlineStr">
         <is>
-          <t>Sentinels</t>
+          <t>Cloud9</t>
         </is>
       </c>
       <c r="D83" s="7" t="n">
-        <v>8</v>
+        <v>7.5</v>
       </c>
       <c r="E83" s="7" t="n">
         <v>6.2</v>
@@ -3664,19 +3664,19 @@
       </c>
       <c r="I83" s="7" t="inlineStr">
         <is>
-          <t>Xeppaa</t>
+          <t>Verno</t>
         </is>
       </c>
       <c r="J83" s="7" t="inlineStr">
         <is>
-          <t>Cloud9</t>
+          <t>MIBR</t>
         </is>
       </c>
       <c r="K83" s="7" t="n">
         <v>8.5</v>
       </c>
       <c r="L83" s="7" t="n">
-        <v>6.2</v>
+        <v>6.9</v>
       </c>
       <c r="M83" s="7" t="inlineStr"/>
     </row>
@@ -3688,19 +3688,19 @@
       </c>
       <c r="B84" s="7" t="inlineStr">
         <is>
-          <t>supamen</t>
+          <t>v1c</t>
         </is>
       </c>
       <c r="C84" s="7" t="inlineStr">
         <is>
-          <t>Evil Geniuses</t>
+          <t>Cloud9</t>
         </is>
       </c>
       <c r="D84" s="7" t="n">
-        <v>6.5</v>
+        <v>8</v>
       </c>
       <c r="E84" s="7" t="n">
-        <v>7.2</v>
+        <v>7</v>
       </c>
       <c r="F84" s="7" t="inlineStr"/>
       <c r="H84" s="6" t="inlineStr">
@@ -3710,19 +3710,19 @@
       </c>
       <c r="I84" s="7" t="inlineStr">
         <is>
-          <t>Erde</t>
+          <t>Veqaj</t>
         </is>
       </c>
       <c r="J84" s="7" t="inlineStr">
         <is>
-          <t>LOUD</t>
+          <t>FNATIC</t>
         </is>
       </c>
       <c r="K84" s="7" t="n">
-        <v>6.5</v>
+        <v>9.5</v>
       </c>
       <c r="L84" s="7" t="n">
-        <v>6.9</v>
+        <v>0</v>
       </c>
       <c r="M84" s="7" t="inlineStr"/>
     </row>
@@ -3734,19 +3734,19 @@
       </c>
       <c r="B85" s="7" t="inlineStr">
         <is>
-          <t>v1c</t>
+          <t>supamen</t>
         </is>
       </c>
       <c r="C85" s="7" t="inlineStr">
         <is>
-          <t>Cloud9</t>
+          <t>Evil Geniuses</t>
         </is>
       </c>
       <c r="D85" s="7" t="n">
-        <v>8</v>
+        <v>6.5</v>
       </c>
       <c r="E85" s="7" t="n">
-        <v>7</v>
+        <v>7.2</v>
       </c>
       <c r="F85" s="7" t="inlineStr"/>
       <c r="H85" s="6" t="inlineStr">
@@ -3756,19 +3756,19 @@
       </c>
       <c r="I85" s="7" t="inlineStr">
         <is>
-          <t>Veqaj</t>
+          <t>Erde</t>
         </is>
       </c>
       <c r="J85" s="7" t="inlineStr">
         <is>
-          <t>FNATIC</t>
+          <t>LOUD</t>
         </is>
       </c>
       <c r="K85" s="7" t="n">
-        <v>9.5</v>
+        <v>6.5</v>
       </c>
       <c r="L85" s="7" t="n">
-        <v>0</v>
+        <v>6.9</v>
       </c>
       <c r="M85" s="7" t="inlineStr"/>
     </row>
@@ -3780,45 +3780,41 @@
       </c>
       <c r="B86" s="7" t="inlineStr">
         <is>
-          <t>Cryocells</t>
+          <t>echo</t>
         </is>
       </c>
       <c r="C86" s="7" t="inlineStr">
         <is>
-          <t>100 Thieves</t>
+          <t>Eternal Fire</t>
         </is>
       </c>
       <c r="D86" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="E86" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F86" s="7" t="inlineStr"/>
+      <c r="H86" s="6" t="inlineStr">
+        <is>
+          <t>S1</t>
+        </is>
+      </c>
+      <c r="I86" s="7" t="inlineStr">
+        <is>
+          <t>Less</t>
+        </is>
+      </c>
+      <c r="J86" s="7" t="inlineStr">
+        <is>
+          <t>KRU Esports</t>
+        </is>
+      </c>
+      <c r="K86" s="7" t="n">
         <v>10.5</v>
       </c>
-      <c r="E86" s="7" t="n">
-        <v>10.5</v>
-      </c>
-      <c r="F86" s="8" t="inlineStr">
-        <is>
-          <t>IGL</t>
-        </is>
-      </c>
-      <c r="H86" s="6" t="inlineStr">
-        <is>
-          <t>S1</t>
-        </is>
-      </c>
-      <c r="I86" s="7" t="inlineStr">
-        <is>
-          <t>skuba</t>
-        </is>
-      </c>
-      <c r="J86" s="7" t="inlineStr">
-        <is>
-          <t>NRG Esports</t>
-        </is>
-      </c>
-      <c r="K86" s="7" t="n">
-        <v>13</v>
-      </c>
       <c r="L86" s="7" t="n">
-        <v>7.5</v>
+        <v>7.4</v>
       </c>
       <c r="M86" s="7" t="inlineStr"/>
     </row>
@@ -3830,19 +3826,19 @@
       </c>
       <c r="B87" s="7" t="inlineStr">
         <is>
-          <t>Less</t>
+          <t>skuba</t>
         </is>
       </c>
       <c r="C87" s="7" t="inlineStr">
         <is>
-          <t>KRU Esports</t>
+          <t>NRG Esports</t>
         </is>
       </c>
       <c r="D87" s="7" t="n">
-        <v>8.5</v>
+        <v>9.5</v>
       </c>
       <c r="E87" s="7" t="n">
-        <v>7.4</v>
+        <v>7.5</v>
       </c>
       <c r="F87" s="7" t="inlineStr"/>
       <c r="H87" s="6" t="inlineStr">
@@ -3876,21 +3872,25 @@
       </c>
       <c r="B88" s="7" t="inlineStr">
         <is>
-          <t>jawgemo</t>
+          <t>dgzin</t>
         </is>
       </c>
       <c r="C88" s="7" t="inlineStr">
         <is>
-          <t>G2 Esports</t>
+          <t>Evil Geniuses</t>
         </is>
       </c>
       <c r="D88" s="7" t="n">
-        <v>13.5</v>
+        <v>11</v>
       </c>
       <c r="E88" s="7" t="n">
-        <v>9.699999999999999</v>
-      </c>
-      <c r="F88" s="7" t="inlineStr"/>
+        <v>10.1</v>
+      </c>
+      <c r="F88" s="8" t="inlineStr">
+        <is>
+          <t>IGL</t>
+        </is>
+      </c>
       <c r="H88" s="6" t="inlineStr">
         <is>
           <t>W1</t>
@@ -3922,19 +3922,19 @@
       </c>
       <c r="B89" s="7" t="inlineStr">
         <is>
-          <t>JohnQT</t>
+          <t>jawgemo</t>
         </is>
       </c>
       <c r="C89" s="7" t="inlineStr">
         <is>
-          <t>Sentinels</t>
+          <t>G2 Esports</t>
         </is>
       </c>
       <c r="D89" s="7" t="n">
-        <v>9</v>
+        <v>13.5</v>
       </c>
       <c r="E89" s="7" t="n">
-        <v>6.7</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="F89" s="7" t="inlineStr"/>
       <c r="H89" s="6" t="inlineStr">
@@ -3944,19 +3944,19 @@
       </c>
       <c r="I89" s="7" t="inlineStr">
         <is>
-          <t>OXY</t>
+          <t>Neon</t>
         </is>
       </c>
       <c r="J89" s="7" t="inlineStr">
         <is>
-          <t>Cloud9</t>
+          <t>LEVIATAN</t>
         </is>
       </c>
       <c r="K89" s="7" t="n">
-        <v>12</v>
+        <v>8.5</v>
       </c>
       <c r="L89" s="7" t="n">
-        <v>7.9</v>
+        <v>10.1</v>
       </c>
       <c r="M89" s="7" t="inlineStr"/>
     </row>
@@ -3968,12 +3968,12 @@
       </c>
       <c r="B90" s="7" t="inlineStr">
         <is>
-          <t>Yetujey</t>
+          <t>xavi8k</t>
         </is>
       </c>
       <c r="C90" s="7" t="inlineStr">
         <is>
-          <t>FUT Esports</t>
+          <t>Global Esports</t>
         </is>
       </c>
       <c r="D90" s="7" t="n">
@@ -3990,19 +3990,19 @@
       </c>
       <c r="I90" s="7" t="inlineStr">
         <is>
-          <t>Autumn</t>
+          <t>OXY</t>
         </is>
       </c>
       <c r="J90" s="7" t="inlineStr">
         <is>
-          <t>Global Esports</t>
+          <t>Cloud9</t>
         </is>
       </c>
       <c r="K90" s="7" t="n">
-        <v>8.5</v>
+        <v>12</v>
       </c>
       <c r="L90" s="7" t="n">
-        <v>0</v>
+        <v>7.9</v>
       </c>
       <c r="M90" s="7" t="inlineStr"/>
     </row>
@@ -4016,11 +4016,11 @@
         <v>100</v>
       </c>
       <c r="E91" s="9" t="n">
-        <v>81.8</v>
+        <v>74.5</v>
       </c>
       <c r="F91" s="5" t="inlineStr">
         <is>
-          <t>IGL: 92.2</t>
+          <t>IGL: 84.7</t>
         </is>
       </c>
       <c r="H91" s="9" t="inlineStr">
@@ -4029,14 +4029,14 @@
         </is>
       </c>
       <c r="J91" s="9" t="n">
-        <v>99.5</v>
+        <v>100</v>
       </c>
       <c r="L91" s="9" t="n">
-        <v>64.7</v>
+        <v>74.7</v>
       </c>
       <c r="M91" s="5" t="inlineStr">
         <is>
-          <t>IGL: 74.8</t>
+          <t>IGL: 84.9</t>
         </is>
       </c>
     </row>

</xml_diff>